<commit_message>
Finished modelling and tunning
</commit_message>
<xml_diff>
--- a/Models.xlsx
+++ b/Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY FILES\IRONHACK\FINAL PROJECT\ai-paper-impact-predictor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7B949B-571B-4F8C-981D-F79ECF256979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1680A1E-1470-434F-89D0-E851C8391A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6C25254-11CD-4CD7-A200-A2193C36F1C2}"/>
   </bookViews>
@@ -209,9 +209,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -221,6 +218,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -268,8 +268,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="14313992" y="7406640"/>
-          <a:ext cx="4701718" cy="5543550"/>
+          <a:off x="14269622" y="7422073"/>
+          <a:ext cx="4686285" cy="5555125"/>
           <a:chOff x="8949512" y="4343400"/>
           <a:chExt cx="4701718" cy="5543550"/>
         </a:xfrm>
@@ -388,8 +388,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9630165" y="7444740"/>
-          <a:ext cx="4695256" cy="5535930"/>
+          <a:off x="9601228" y="7460173"/>
+          <a:ext cx="4679823" cy="5547505"/>
           <a:chOff x="4136145" y="4396740"/>
           <a:chExt cx="4695256" cy="5535930"/>
         </a:xfrm>
@@ -508,8 +508,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4937760" y="7444740"/>
-          <a:ext cx="4693813" cy="8976360"/>
+          <a:off x="4922327" y="7460173"/>
+          <a:ext cx="4680309" cy="8995265"/>
           <a:chOff x="4202536" y="2011680"/>
           <a:chExt cx="4693813" cy="8976360"/>
         </a:xfrm>
@@ -634,8 +634,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="68580" y="7498080"/>
-          <a:ext cx="4688793" cy="5528310"/>
+          <a:off x="68580" y="7513899"/>
+          <a:ext cx="4675289" cy="5539884"/>
           <a:chOff x="1304336" y="5036820"/>
           <a:chExt cx="4688793" cy="5528310"/>
         </a:xfrm>
@@ -1190,13 +1190,13 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
@@ -1219,118 +1219,118 @@
       <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <v>6.4210000000000003</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <v>5.5629999999999997</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <v>6.3049999999999997</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="6">
         <v>6.8029999999999999</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <v>4.1390000000000002</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <v>4.9969999999999999</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <v>4.2549999999999999</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <v>3.7570000000000001</v>
       </c>
     </row>

</xml_diff>